<commit_message>
Send mobile users to the right tab after email, password, and OTP login.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -890,9 +890,9 @@
           <t>screens/auth/LoginScreen.jsx</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Customer and vendor log in and land on the right tabs.</t>
+          <t>Customer lands on Home. Vendor lands on the vendor tab. OTP is required after the password, same as the website.</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Screen exists. Retest on a device with live SMS.</t>
+          <t>Forgot password is row 13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify new customer accounts with a phone OTP and open Home after signup.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -942,9 +942,9 @@
           <t>screens/auth/RegisterScreen.jsx</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -959,10 +959,14 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>New customer account is created and the phone OTP verifies.</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr"/>
+          <t>Name, email, 10-digit phone, and password create the account. Phone OTP verifies it and opens Home.</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Password must match and be at least 6 characters, same as the website.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Open the vendor tab after vendor signup and phone OTP.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -994,9 +994,9 @@
           <t>screens/auth/VendorRegisterScreen.jsx</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -1011,10 +1011,14 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Vendor account is created and opens the vendor tab.</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr"/>
+          <t>Vendor picks a business type, verifies the phone OTP, then opens the vendor tab. Shop vendors open KYC.</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Creating the listing form is a later row. Driver and shop types are included.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add a forgot-password screen to the mobile login flow.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1043,12 +1043,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>screens/auth/ForgotPasswordScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1063,10 +1063,14 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>User can request a reset from the login screen.</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr"/>
+          <t>From login, the user enters an email and the app requests a password reset, same as the website.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>The email is sent only after SMTP is configured.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Add the Drivers tile to the mobile home category grid.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1098,9 +1098,9 @@
           <t>screens/customer/HomeScreen.jsx</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1115,12 +1115,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Tiles for hotels, resorts, homestays, tents, guides, taxi, drivers, horses, strawberries, Mapro, and combos.</t>
+          <t>Home shows hotels, resorts, homestays, tents, guides, drivers, taxi, horses, strawberries, Mapro, and combos.</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Drivers tile is missing.</t>
+          <t>Drivers tile opens the driver catalog. The dedicated driver booking flow is a later row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show hotel photos, price, location, and rooms on the mobile listing screens.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1150,9 +1150,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Photos, price, location, and rooms match the website data.</t>
+          <t>Hotel list and detail show the photo, price, location, and rooms from the same API as the website.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Generic list, not the website layout.</t>
+          <t>The full guest booking form is a later row. The chosen room is sent with the booking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
List resorts as a hotel filter and show the same stay details.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1202,9 +1202,9 @@
           <t>CatalogScreen.jsx</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1219,10 +1219,14 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Resorts are a filter on hotels, same as the website.</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr"/>
+          <t>Resorts are hotels filtered by type RESORT. Detail shows photo, price, location, and rooms.</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Same screens as hotels. An empty resort list says nothing is here, not an error.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Show homestay photos, nightly price, facilities, and stay rules.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1254,9 +1254,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1271,10 +1271,14 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Stay details and price match the website.</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr"/>
+          <t>Homestay list and detail show photo, nightly price, location, facilities, check-in times, house rules, and rooms.</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Guest registration form is row 29. The selected room is sent with the booking.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Show tent capacity, nightly price, facilities, and stay rules.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1306,9 +1306,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1323,10 +1323,14 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Tent details match the website.</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr"/>
+          <t>Tent list and detail show photo, nightly price, location, capacity, facilities, and check-in rules.</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>The tent guest booking form is row 30.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Show guide package prices and the official rate chart before booking.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1358,9 +1358,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Guide packages are visible before booking.</t>
+          <t>Guide list shows the 6-hour price. Detail shows this guide packages plus the official rate chart and sightseeing points.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Detail page does not show the website rate chart.</t>
+          <t>The full guide booking form is row 31. The selected 6hr or 12hr package and bike add-on are sent with the booking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show taxi car types and route fares before booking.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1410,9 +1410,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1427,10 +1427,14 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Routes and car types are visible before booking.</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr"/>
+          <t>Taxi list loads taxi operators and shows car types plus local and outstation routes before booking.</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>The full taxi guest form is row 32. The selected car, route, and per-trip or hourly fare are sent with the booking.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Open drivers into a booking entry with the website package prices.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1459,12 +1459,12 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1479,12 +1479,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Drivers appear in the home grid and open a driver booking flow.</t>
+          <t>Drivers tile opens driver partners plus the booking entry: how it works and the 4hr, 8hr, and 12hr packages.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Not in mobile CATEGORIES.</t>
+          <t>The full driver guest form is row 33. The selected package is sent with the booking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show horse ride packages and stable routes before booking.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1514,9 +1514,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1531,10 +1531,14 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Horse packages are visible before booking.</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr"/>
+          <t>Horse list and detail show the official ride packages plus each stable routes, duration, and price.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>The full horse guest form is row 34. The selected route is sent with the booking.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Show strawberry photos, descriptions, and prices on the shop list.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1566,9 +1566,9 @@
           <t>CatalogScreen.jsx</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1583,10 +1583,14 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Strawberry products list with price and photo.</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr"/>
+          <t>Strawberry products list shows the photo, short description, price, and unit from the same products API as the website.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Ordering with quantity is row 35.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Show Mapro photos, descriptions, and prices on the shop list.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1618,9 +1618,9 @@
           <t>CatalogScreen.jsx</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1635,10 +1635,14 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Mapro products list with price and photo.</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr"/>
+          <t>Mapro products list shows the photo, short description, price, and unit from the same products API as the website.</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>Ordering with quantity is row 35.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Book horse rides from the official package chart.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -1670,9 +1670,9 @@
           <t>CatalogScreen.jsx, ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1687,10 +1687,14 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Combo contents and price match the website.</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr"/>
+          <t>Combo list and detail show the photo, description, included items, combo price, original price, and savings.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Choosing the stay date and confirming the booking is row 36.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1715,12 +1719,12 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>screens/customer/SearchScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1735,10 +1739,14 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Search finds listings across services.</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr"/>
+          <t>Home search uses the same /search API as the website and groups hotels, resorts, homestays, tents, guides, taxis, drivers, and horses.</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Products and combos are not in the website search API.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -1763,12 +1771,12 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>screens/customer/ContentScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1783,12 +1791,12 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Static pages open inside the app.</t>
+          <t>Account opens About, contact, FAQ, blogs, About Mahabaleshwar, privacy, terms, and cancellation inside the app.</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Do these after booking works.</t>
+          <t>FAQ and blogs use the public API. Contact posts the same general enquiry as the website.</t>
         </is>
       </c>
     </row>
@@ -1818,9 +1826,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1835,12 +1843,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Dates, guests, and room choice create the same booking as the website.</t>
+          <t>Hotel and resort booking sends the selected room, check-in, check-out, adults, children, lead guest, and ID, and shows the night total.</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Current form always uses the first room.</t>
+          <t>Payment checkout is row 37.</t>
         </is>
       </c>
     </row>
@@ -1870,9 +1878,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1887,10 +1895,14 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Dates and guests match the website rules.</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr"/>
+          <t>Homestay booking sends the selected room, check-in, check-out, adults, children, lead guest, and ID, and shows the night total.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Payment checkout is row 37.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -1918,9 +1930,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1935,10 +1947,14 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Tent dates and guest count match the website.</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr"/>
+          <t>Tent booking sends check-in, check-out, tent count, adults, children, lead guest, and ID, and shows the night total.</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>Payment checkout is row 37.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -1966,9 +1982,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1983,12 +1999,12 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Package, bike add-on, and price match the website rate chart.</t>
+          <t>Guide booking uses the official 4-hour and 8-hour chart. Bike add-on changes the price to 1100 or 1700, and the request stores that total.</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>App currently sends a fixed 6-hour package.</t>
+          <t>Same as the website open guide form: a guide is assigned later. Payment is row 37.</t>
         </is>
       </c>
     </row>
@@ -2018,9 +2034,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -2035,12 +2051,12 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Route, car type, and price match the website.</t>
+          <t>Taxi booking sends the selected chart route, car type, and that route price, plus the trip date, pickup, and guest contact.</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>App currently sends a fixed TRIP type.</t>
+          <t>Same as the website open taxi form: a taxi is assigned later. Payment is row 37.</t>
         </is>
       </c>
     </row>
@@ -2067,12 +2083,12 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>ListingDetailScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2087,10 +2103,14 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Driver package and price match the website.</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr"/>
+          <t>Driver booking sends the selected 4-hour, 8-hour, or 12-hour package and that chart price, plus the trip date, pickup, and guest contact.</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Same as the website open driver form: a driver is assigned later. Payment is row 37.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -2118,9 +2138,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2135,10 +2155,14 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Package and price match the website.</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr"/>
+          <t>Horse booking sends the selected official package and that chart price, plus the ride date, rider count, guest contact, and safety confirmation.</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>Same as the website open horse form: a stable is assigned later. Payment is row 37. Stable route prices still show on the detail screen.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Let vendors mark arrival and propose the end with overtime.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -2190,9 +2190,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2207,10 +2207,14 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Quantity and total match the website.</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr"/>
+          <t>Product order sends the quantity and shows the line total (price times quantity), with the same local delivery note as the website.</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Payment checkout is row 37.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -2238,9 +2242,9 @@
           <t>ListingDetailScreen.jsx</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2255,10 +2259,14 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Date and price match the website.</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="inlineStr"/>
+          <t>Combo booking sends the check-in date and stores the combo price. The form shows that price, the struck original price, and the included items.</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>Payment checkout is row 37. Guest count stays the API default of 2 adults, same as the website.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2286,9 +2294,9 @@
           <t>screens/customer/BookingsScreen.jsx</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2303,12 +2311,12 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Customer pays with the live Razorpay key and the booking is marked paid.</t>
+          <t>Pay now opens Razorpay checkout with the live key and verifies the returned signature, which marks the booking paid.</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>App still verifies a mock payment.</t>
+          <t>Mock verify remains only when the API returns a mock order. Reload the Expo app after this change.</t>
         </is>
       </c>
     </row>
@@ -2338,9 +2346,9 @@
           <t>screens/customer/BookingsScreen.jsx</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -2355,10 +2363,14 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>List, status, invoice, and refund request match the website.</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr"/>
+          <t>Bookings list shows the listing name, status, date, and total. Invoice downloads with the signed-in account. Refund shows the estimated amount before it is sent.</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Reload Expo after this change. Reviews are a later row.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2386,9 +2398,9 @@
           <t>screens/customer/BookingsScreen.jsx</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2403,12 +2415,12 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Customer can confirm arrival and service end, including overtime.</t>
+          <t>Customer confirms partner arrival, then confirms the end. Overtime hours and amount are shown before the end is confirmed, and the invoice can be downloaded after.</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Buttons exist. Recheck against the website.</t>
+          <t>Partner marks arrival and proposes the end. Those vendor actions stay on the vendor booking rows.</t>
         </is>
       </c>
     </row>
@@ -2438,9 +2450,9 @@
           <t>screens/customer/AccountScreen.jsx</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -2455,12 +2467,12 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>Name, email, and phone can be updated.</t>
+          <t>Account lets the signed-in user edit name, email, and phone, then saves them on the profile.</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>View only today.</t>
+          <t>Email must stay unique. The website form still edits name and phone only.</t>
         </is>
       </c>
     </row>
@@ -2487,12 +2499,12 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>FavoritesScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2510,7 +2522,11 @@
           <t>Customer can save and reopen a listing.</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Save on the listing. Reopen from Account, Saved listings.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
@@ -2538,9 +2554,9 @@
           <t>screens/vendor/VendorHubScreen.jsx</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2560,7 +2576,7 @@
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>No purchase or payout history.</t>
+          <t>Hub shows wallet balance, point balance, and the active plan with its end date.</t>
         </is>
       </c>
     </row>
@@ -2590,9 +2606,9 @@
           <t>screens/vendor/VendorKycScreen.jsx</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2612,7 +2628,7 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>No document photo upload yet.</t>
+          <t>Aadhaar, PAN, GST, and bank details load and submit. Document photos stay on the website.</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2655,12 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorListingsScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2662,7 +2678,11 @@
           <t>Vendor sees only their own listings for their role.</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr"/>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>Each role loads only its own /mine listings, with status and from-price.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -2687,12 +2707,12 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorListingFormScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2710,7 +2730,11 @@
           <t>Create and edit match the website form for that vendor role.</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Create and edit use the same fields and payload as the website for that role. Approved listings can be edited.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
@@ -2735,12 +2759,12 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorPricingScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2758,7 +2782,11 @@
           <t>Price changes save and show on the customer listing.</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr"/>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>Vendor saves room, package, trip, route, or product prices. The public listing uses those prices.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -2783,12 +2811,12 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorAvailabilityScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2808,7 +2836,7 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>Only roles that have availability on the website.</t>
+          <t>Vendor blocks or opens a day. Booked and past days stay locked. Booking rejects a blocked date.</t>
         </is>
       </c>
     </row>
@@ -2838,9 +2866,9 @@
           <t>screens/customer/BookingsScreen.jsx</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -2860,7 +2888,7 @@
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>Shared with the customer bookings screen.</t>
+          <t>Vendor marks arrival, then proposes the end with overtime hours at Rs 150 per hour.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Let hotel, homestay, and tent vendors buy a homepage ad.
</commit_message>
<xml_diff>
--- a/docs/Mobile_App_Implementation_Tracker.xlsx
+++ b/docs/Mobile_App_Implementation_Tracker.xlsx
@@ -2915,12 +2915,12 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorReviewsScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2938,7 +2938,11 @@
           <t>Vendor can read reviews on their listings.</t>
         </is>
       </c>
-      <c r="J49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Vendor reads guest reviews for their own listings, with rating, comment, and booking number.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
@@ -2963,12 +2967,12 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>screens/vendor/VendorHubScreen.jsx</t>
-        </is>
-      </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorHubScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -2988,7 +2992,7 @@
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>Hub shows balance only.</t>
+          <t>Vendor buys points at the recharge rate and sees the latest wallet transactions.</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3019,12 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>screens/vendor/VendorHubScreen.jsx</t>
-        </is>
-      </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorSubscriptionScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -3040,7 +3044,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Hub shows status only.</t>
+          <t>Stay listings renew through Razorpay. Service vendors recharge points or buy the unlimited month the same way.</t>
         </is>
       </c>
     </row>
@@ -3067,12 +3071,12 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>VendorAdsScreen.jsx</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -3090,7 +3094,11 @@
           <t>Vendor can buy a homepage ad the same way as the website.</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr"/>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>Hotel, homestay, and tent vendors pay for a homepage spotlight on an approved listing and see their ad history.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="4" t="inlineStr">

</xml_diff>